<commit_message>
Build Starter City route-map campaign
</commit_message>
<xml_diff>
--- a/outputs/card_inventory_2026-07-18/topdeck_to_worlds_implemented_cards.xlsx
+++ b/outputs/card_inventory_2026-07-18/topdeck_to_worlds_implemented_cards.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R260e59ec89fe481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="Ra5052fdb28b04c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Starter Decks" sheetId="3" r:id="R45d8a44ed8d348eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Raa31f002e9d1465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cards" sheetId="2" r:id="R6768309254824a9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Starter Decks" sheetId="3" r:id="R8052fa25b93748aa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1769,7 +1769,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="16" t="str">
-        <x:v>Topdeck to Worlds — Implemented Card Catalog</x:v>
+        <x:v>TOP CUT: Locals to Worlds — Implemented Card Catalog</x:v>
       </x:c>
       <x:c r="B1" s="16"/>
       <x:c r="C1" s="16"/>
@@ -7387,7 +7387,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d923ff9c950477c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88695acf4d9b4e1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9090,7 +9090,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8c7d73878624bd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14a00c4322054a88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>